<commit_message>
completed prelim analyses of HMPV+RSV circulation
</commit_message>
<xml_diff>
--- a/Data/nvsn_PITT_ANNA_HMPV_DD_12.19.25.xlsx
+++ b/Data/nvsn_PITT_ANNA_HMPV_DD_12.19.25.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\cdc.gov\project\NCIRD_DVD_EB_NVSN2\ARI\Personal Folders\Leah\Data requests\Site data requests\Datasets and DDs\DDs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://pitt-my.sharepoint.com/personal/rdp57_pitt_edu/Documents/Documents/R/HMPV Co-detections/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B8A60F8-8249-47CF-97B1-EA9247BC24F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1385,17 +1385,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E53"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="21.140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="52.85546875" style="1" customWidth="1"/>
-    <col min="4" max="4" width="137.5703125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="67.85546875" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="21.109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="52.88671875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="137.5546875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="67.88671875" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="9" t="s">
         <v>28</v>
       </c>
@@ -1404,14 +1404,14 @@
       <c r="D1" s="9"/>
       <c r="E1" s="9"/>
     </row>
-    <row r="2" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9"/>
       <c r="B2" s="9"/>
       <c r="C2" s="9"/>
       <c r="D2" s="9"/>
       <c r="E2" s="9"/>
     </row>
-    <row r="3" spans="1:5" s="7" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" s="7" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>0</v>
       </c>
@@ -1428,7 +1428,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>29</v>
       </c>
@@ -1437,7 +1437,7 @@
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
@@ -1451,7 +1451,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>33</v>
       </c>
@@ -1465,7 +1465,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
@@ -1479,7 +1479,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>8</v>
       </c>
@@ -1493,7 +1493,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>36</v>
       </c>
@@ -1510,7 +1510,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>39</v>
       </c>
@@ -1524,7 +1524,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
@@ -1538,7 +1538,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="8" t="s">
         <v>30</v>
       </c>
@@ -1547,7 +1547,7 @@
       <c r="D12" s="8"/>
       <c r="E12" s="8"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>45</v>
       </c>
@@ -1561,7 +1561,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>47</v>
       </c>
@@ -1575,7 +1575,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>49</v>
       </c>
@@ -1589,7 +1589,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>53</v>
       </c>
@@ -1606,7 +1606,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>56</v>
       </c>
@@ -1623,7 +1623,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>60</v>
       </c>
@@ -1640,7 +1640,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
         <v>31</v>
       </c>
@@ -1649,7 +1649,7 @@
       <c r="D19" s="8"/>
       <c r="E19" s="8"/>
     </row>
-    <row r="20" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>83</v>
       </c>
@@ -1666,7 +1666,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>86</v>
       </c>
@@ -1683,7 +1683,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>92</v>
       </c>
@@ -1700,7 +1700,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>89</v>
       </c>
@@ -1717,7 +1717,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>98</v>
       </c>
@@ -1734,7 +1734,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
         <v>101</v>
       </c>
@@ -1751,7 +1751,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
         <v>102</v>
       </c>
@@ -1768,7 +1768,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="8" t="s">
         <v>32</v>
       </c>
@@ -1777,7 +1777,7 @@
       <c r="D27" s="8"/>
       <c r="E27" s="8"/>
     </row>
-    <row r="28" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
         <v>95</v>
       </c>
@@ -1791,7 +1791,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
         <v>96</v>
       </c>
@@ -1805,7 +1805,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>20</v>
       </c>
@@ -1819,7 +1819,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
         <v>97</v>
       </c>
@@ -1833,7 +1833,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>16</v>
       </c>
@@ -1847,7 +1847,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>19</v>
       </c>
@@ -1864,7 +1864,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
         <v>108</v>
       </c>
@@ -1881,7 +1881,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>110</v>
       </c>
@@ -1898,7 +1898,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
         <v>113</v>
       </c>
@@ -1915,7 +1915,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
         <v>115</v>
       </c>
@@ -1932,7 +1932,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
         <v>118</v>
       </c>
@@ -1946,7 +1946,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>25</v>
       </c>
@@ -1963,7 +1963,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>21</v>
       </c>
@@ -1980,7 +1980,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="8" t="s">
         <v>63</v>
       </c>
@@ -1989,7 +1989,7 @@
       <c r="D41" s="8"/>
       <c r="E41" s="8"/>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>64</v>
       </c>
@@ -2003,7 +2003,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>66</v>
       </c>
@@ -2017,7 +2017,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>68</v>
       </c>
@@ -2031,7 +2031,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
         <v>70</v>
       </c>
@@ -2045,7 +2045,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
         <v>72</v>
       </c>
@@ -2059,7 +2059,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
         <v>75</v>
       </c>
@@ -2073,7 +2073,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
         <v>78</v>
       </c>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="E48" s="3"/>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>80</v>
       </c>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="E49" s="4"/>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="8" t="s">
         <v>103</v>
       </c>
@@ -2112,7 +2112,7 @@
       <c r="D50" s="8"/>
       <c r="E50" s="8"/>
     </row>
-    <row r="51" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>106</v>
       </c>
@@ -2129,7 +2129,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>107</v>
       </c>
@@ -2146,7 +2146,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>104</v>
       </c>

</xml_diff>